<commit_message>
072425 - updated week 11 skins
</commit_message>
<xml_diff>
--- a/public/results/2025/Week 12 Skins.xlsx
+++ b/public/results/2025/Week 12 Skins.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\CODE\golf-league-site\public\results\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE5EC74-2958-724B-A265-7AF3174A184B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382C94B9-7C59-4F56-9BDD-49ABD9FF6CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3920" yWindow="720" windowWidth="28800" windowHeight="19700" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
+    <workbookView xWindow="555" yWindow="390" windowWidth="19470" windowHeight="10755" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
   </bookViews>
   <sheets>
-    <sheet name="Week 10 Skins" sheetId="1" r:id="rId1"/>
+    <sheet name="Week 12 Skins" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="19">
   <si>
     <t>Skins Won</t>
   </si>
@@ -80,19 +80,7 @@
     <t>Aaron</t>
   </si>
   <si>
-    <t>Kevin</t>
-  </si>
-  <si>
-    <t>Randy</t>
-  </si>
-  <si>
-    <t>Jon</t>
-  </si>
-  <si>
     <t>Matt</t>
-  </si>
-  <si>
-    <t>Jeff</t>
   </si>
   <si>
     <t>Tony</t>
@@ -101,10 +89,10 @@
     <t>Mike W</t>
   </si>
   <si>
-    <t>Mike G</t>
+    <t>John</t>
   </si>
   <si>
-    <t>John</t>
+    <t>Shayne I</t>
   </si>
 </sst>
 </file>
@@ -114,7 +102,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -165,21 +153,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -550,7 +523,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -654,11 +627,23 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -674,54 +659,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1058,33 +995,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F8EC831-685C-42E6-9510-7BA05FCAF636}">
-  <dimension ref="A1:O46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:O31"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.5" style="23" customWidth="1"/>
-    <col min="2" max="2" width="6.5" style="23" customWidth="1"/>
-    <col min="3" max="11" width="8.6640625" style="23" customWidth="1"/>
-    <col min="12" max="12" width="3.1640625" style="23" customWidth="1"/>
-    <col min="13" max="13" width="5.5" style="23" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.33203125" style="23" customWidth="1"/>
-    <col min="15" max="15" width="6.83203125" style="23" customWidth="1"/>
-    <col min="16" max="16384" width="9.1640625" style="23"/>
+    <col min="1" max="1" width="9.42578125" style="23" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125" style="23" customWidth="1"/>
+    <col min="3" max="11" width="8.7109375" style="23" customWidth="1"/>
+    <col min="12" max="12" width="3.140625" style="23" customWidth="1"/>
+    <col min="13" max="13" width="5.42578125" style="23" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.28515625" style="23" customWidth="1"/>
+    <col min="15" max="15" width="6.85546875" style="23" customWidth="1"/>
+    <col min="16" max="16384" width="9.140625" style="23"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>0</v>
@@ -1094,7 +1031,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="24" t="s">
         <v>2</v>
       </c>
@@ -1128,14 +1065,14 @@
       <c r="K2" s="6">
         <v>9</v>
       </c>
-      <c r="L2" s="39" t="s">
+      <c r="L2" s="43" t="s">
         <v>7</v>
       </c>
       <c r="M2" s="7"/>
       <c r="N2" s="8"/>
       <c r="O2" s="9"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="25"/>
       <c r="B3" s="10" t="s">
         <v>4</v>
@@ -1167,12 +1104,12 @@
       <c r="K3" s="11">
         <v>5</v>
       </c>
-      <c r="L3" s="40"/>
+      <c r="L3" s="44"/>
       <c r="M3" s="12"/>
       <c r="N3" s="13"/>
       <c r="O3" s="13"/>
     </row>
-    <row r="4" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="26"/>
       <c r="B4" s="14" t="s">
         <v>7</v>
@@ -1204,13 +1141,13 @@
       <c r="K4" s="15">
         <v>2</v>
       </c>
-      <c r="L4" s="41"/>
+      <c r="L4" s="45"/>
       <c r="M4" s="12"/>
       <c r="N4" s="13"/>
       <c r="O4" s="13"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="42" t="s">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="35" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="28" t="s">
@@ -1248,34 +1185,34 @@
       <c r="N5" s="18"/>
       <c r="O5" s="13"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="43"/>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="31"/>
       <c r="B6" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="46">
-        <v>1</v>
-      </c>
-      <c r="D6" s="46">
-        <v>1</v>
-      </c>
-      <c r="E6" s="46">
-        <v>1</v>
-      </c>
-      <c r="F6" s="46"/>
-      <c r="G6" s="46">
-        <v>1</v>
-      </c>
-      <c r="H6" s="46">
-        <v>1</v>
-      </c>
-      <c r="I6" s="46">
-        <v>1</v>
-      </c>
-      <c r="J6" s="46">
-        <v>1</v>
-      </c>
-      <c r="K6" s="47">
+      <c r="C6" s="36">
+        <v>1</v>
+      </c>
+      <c r="D6" s="36">
+        <v>1</v>
+      </c>
+      <c r="E6" s="36">
+        <v>1</v>
+      </c>
+      <c r="F6" s="36"/>
+      <c r="G6" s="36">
+        <v>1</v>
+      </c>
+      <c r="H6" s="36">
+        <v>1</v>
+      </c>
+      <c r="I6" s="36">
+        <v>1</v>
+      </c>
+      <c r="J6" s="36">
+        <v>1</v>
+      </c>
+      <c r="K6" s="37">
         <v>1</v>
       </c>
       <c r="L6" s="16">
@@ -1286,24 +1223,24 @@
       <c r="N6" s="18"/>
       <c r="O6" s="13"/>
     </row>
-    <row r="7" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="44"/>
+    <row r="7" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="27"/>
       <c r="B7" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="48">
+      <c r="C7" s="38">
         <f>C5-C6</f>
         <v>4</v>
       </c>
-      <c r="D7" s="48">
+      <c r="D7" s="38">
         <f t="shared" ref="D7:K7" si="0">D5-D6</f>
         <v>8</v>
       </c>
-      <c r="E7" s="48">
+      <c r="E7" s="38">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="F7" s="48">
+      <c r="F7" s="38">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
@@ -1311,19 +1248,19 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="H7" s="48">
+      <c r="H7" s="38">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="I7" s="48">
+      <c r="I7" s="38">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="J7" s="48">
+      <c r="J7" s="38">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="K7" s="49">
+      <c r="K7" s="39">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -1332,8 +1269,8 @@
       <c r="N7" s="18"/>
       <c r="O7" s="13"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="42" t="s">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="35" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="28" t="s">
@@ -1371,36 +1308,36 @@
       <c r="N8" s="18"/>
       <c r="O8" s="13"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="43"/>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="31"/>
       <c r="B9" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="46">
-        <v>1</v>
-      </c>
-      <c r="D9" s="46">
-        <v>1</v>
-      </c>
-      <c r="E9" s="46">
-        <v>1</v>
-      </c>
-      <c r="F9" s="46">
-        <v>1</v>
-      </c>
-      <c r="G9" s="46">
-        <v>1</v>
-      </c>
-      <c r="H9" s="46">
-        <v>1</v>
-      </c>
-      <c r="I9" s="46">
-        <v>1</v>
-      </c>
-      <c r="J9" s="46">
-        <v>1</v>
-      </c>
-      <c r="K9" s="47">
+      <c r="C9" s="36">
+        <v>1</v>
+      </c>
+      <c r="D9" s="36">
+        <v>1</v>
+      </c>
+      <c r="E9" s="36">
+        <v>1</v>
+      </c>
+      <c r="F9" s="36">
+        <v>1</v>
+      </c>
+      <c r="G9" s="36">
+        <v>1</v>
+      </c>
+      <c r="H9" s="36">
+        <v>1</v>
+      </c>
+      <c r="I9" s="36">
+        <v>1</v>
+      </c>
+      <c r="J9" s="36">
+        <v>1</v>
+      </c>
+      <c r="K9" s="37">
         <v>1</v>
       </c>
       <c r="L9" s="16">
@@ -1411,44 +1348,44 @@
       <c r="N9" s="18"/>
       <c r="O9" s="13"/>
     </row>
-    <row r="10" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="44"/>
+    <row r="10" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="27"/>
       <c r="B10" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="48">
+      <c r="C10" s="38">
         <f>C8-C9</f>
         <v>6</v>
       </c>
-      <c r="D10" s="48">
+      <c r="D10" s="38">
         <f t="shared" ref="D10:K10" si="1">D8-D9</f>
         <v>5</v>
       </c>
-      <c r="E10" s="48">
+      <c r="E10" s="38">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="F10" s="48">
+      <c r="F10" s="38">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="G10" s="48">
+      <c r="G10" s="38">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="H10" s="48">
+      <c r="H10" s="38">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="I10" s="48">
+      <c r="I10" s="38">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="J10" s="48">
+      <c r="J10" s="38">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="K10" s="57">
+      <c r="K10" s="40">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -1457,359 +1394,371 @@
       <c r="N10" s="18"/>
       <c r="O10" s="13"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="42" t="s">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="35" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="28" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D11" s="32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E11" s="32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F11" s="32">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G11" s="32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H11" s="32">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I11" s="32">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J11" s="32">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K11" s="32">
-        <v>6</v>
-      </c>
-      <c r="L11" s="22"/>
+        <v>5</v>
+      </c>
+      <c r="L11" s="16"/>
       <c r="M11" s="17"/>
       <c r="N11" s="18"/>
       <c r="O11" s="13"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="43"/>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="31"/>
       <c r="B12" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="46">
-        <v>2</v>
-      </c>
-      <c r="D12" s="46">
-        <v>3</v>
-      </c>
-      <c r="E12" s="46">
-        <v>2</v>
-      </c>
-      <c r="F12" s="46">
-        <v>2</v>
-      </c>
-      <c r="G12" s="46">
-        <v>2</v>
-      </c>
-      <c r="H12" s="46">
-        <v>2</v>
-      </c>
-      <c r="I12" s="46">
-        <v>2</v>
-      </c>
-      <c r="J12" s="46">
-        <v>2</v>
-      </c>
-      <c r="K12" s="47">
-        <v>2</v>
+      <c r="C12" s="36">
+        <v>1</v>
+      </c>
+      <c r="D12" s="36">
+        <v>1</v>
+      </c>
+      <c r="E12" s="36">
+        <v>1</v>
+      </c>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36">
+        <v>1</v>
+      </c>
+      <c r="H12" s="36">
+        <v>1</v>
+      </c>
+      <c r="I12" s="36">
+        <v>1</v>
+      </c>
+      <c r="J12" s="36">
+        <v>1</v>
+      </c>
+      <c r="K12" s="37">
+        <v>1</v>
       </c>
       <c r="L12" s="16">
         <f>SUM(C12:K12)</f>
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="M12" s="17"/>
       <c r="N12" s="18"/>
       <c r="O12" s="13"/>
     </row>
-    <row r="13" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="44"/>
+    <row r="13" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="27"/>
       <c r="B13" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="34">
+      <c r="C13" s="38">
         <f>C11-C12</f>
-        <v>3</v>
-      </c>
-      <c r="D13" s="48">
+        <v>5</v>
+      </c>
+      <c r="D13" s="38">
         <f t="shared" ref="D13:K13" si="2">D11-D12</f>
-        <v>4</v>
-      </c>
-      <c r="E13" s="48">
+        <v>5</v>
+      </c>
+      <c r="E13" s="38">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="F13" s="48">
+      <c r="F13" s="34">
         <f t="shared" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="G13" s="48">
+        <v>2</v>
+      </c>
+      <c r="G13" s="34">
         <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="H13" s="48">
+        <v>3</v>
+      </c>
+      <c r="H13" s="38">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="I13" s="48">
+      <c r="I13" s="38">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="J13" s="48">
+      <c r="J13" s="38">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="K13" s="49">
+      <c r="K13" s="38">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
       <c r="L13" s="19"/>
-      <c r="M13" s="17"/>
+      <c r="M13" s="20"/>
       <c r="N13" s="18"/>
-      <c r="O13" s="13"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="42" t="s">
+      <c r="O13" s="21"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="35" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="28" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="32">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D14" s="32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E14" s="32">
         <v>5</v>
       </c>
       <c r="F14" s="32">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G14" s="32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H14" s="32">
         <v>5</v>
       </c>
       <c r="I14" s="32">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J14" s="32">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K14" s="32">
-        <v>7</v>
-      </c>
-      <c r="L14" s="22"/>
+        <v>6</v>
+      </c>
+      <c r="L14" s="16"/>
       <c r="M14" s="17"/>
       <c r="N14" s="18"/>
       <c r="O14" s="13"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="43"/>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="31"/>
       <c r="B15" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="46">
-        <v>2</v>
-      </c>
-      <c r="D15" s="46">
-        <v>2</v>
-      </c>
-      <c r="E15" s="46">
-        <v>2</v>
-      </c>
-      <c r="F15" s="46">
-        <v>1</v>
-      </c>
-      <c r="G15" s="46">
-        <v>1</v>
-      </c>
-      <c r="H15" s="46">
-        <v>1</v>
-      </c>
-      <c r="I15" s="46">
-        <v>1</v>
-      </c>
-      <c r="J15" s="46">
-        <v>1</v>
-      </c>
-      <c r="K15" s="47">
+      <c r="C15" s="36">
+        <v>1</v>
+      </c>
+      <c r="D15" s="36">
+        <v>2</v>
+      </c>
+      <c r="E15" s="36">
+        <v>2</v>
+      </c>
+      <c r="F15" s="36">
+        <v>1</v>
+      </c>
+      <c r="G15" s="36">
+        <v>1</v>
+      </c>
+      <c r="H15" s="36">
+        <v>1</v>
+      </c>
+      <c r="I15" s="36">
+        <v>1</v>
+      </c>
+      <c r="J15" s="36">
+        <v>1</v>
+      </c>
+      <c r="K15" s="37">
         <v>2</v>
       </c>
       <c r="L15" s="16">
         <f>SUM(C15:K15)</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M15" s="17"/>
       <c r="N15" s="18"/>
       <c r="O15" s="13"/>
     </row>
-    <row r="16" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="44"/>
+    <row r="16" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="27"/>
       <c r="B16" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="48">
+      <c r="C16" s="38">
         <f>C14-C15</f>
         <v>4</v>
       </c>
-      <c r="D16" s="48">
+      <c r="D16" s="38">
         <f t="shared" ref="D16:K16" si="3">D14-D15</f>
-        <v>3</v>
-      </c>
-      <c r="E16" s="48">
+        <v>4</v>
+      </c>
+      <c r="E16" s="38">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="F16" s="48">
+      <c r="F16" s="38">
         <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-      <c r="G16" s="48">
+        <v>4</v>
+      </c>
+      <c r="G16" s="34">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="H16" s="48">
+        <v>3</v>
+      </c>
+      <c r="H16" s="38">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="I16" s="48">
+      <c r="I16" s="38">
         <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="J16" s="48">
+        <v>2</v>
+      </c>
+      <c r="J16" s="38">
         <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="K16" s="49">
+        <v>4</v>
+      </c>
+      <c r="K16" s="38">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L16" s="19"/>
-      <c r="M16" s="17"/>
+      <c r="M16" s="20"/>
       <c r="N16" s="18"/>
-      <c r="O16" s="13"/>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="42" t="s">
-        <v>16</v>
+      <c r="O16" s="21"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="35" t="s">
+        <v>5</v>
       </c>
       <c r="B17" s="28" t="s">
         <v>8</v>
       </c>
       <c r="C17" s="32">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D17" s="32">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E17" s="32">
-        <v>4</v>
-      </c>
-      <c r="F17" s="45">
-        <v>2</v>
-      </c>
-      <c r="G17" s="45">
-        <v>5</v>
-      </c>
-      <c r="H17" s="45">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="F17" s="32">
+        <v>3</v>
+      </c>
+      <c r="G17" s="32">
+        <v>8</v>
+      </c>
+      <c r="H17" s="32">
+        <v>6</v>
       </c>
       <c r="I17" s="32">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J17" s="32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K17" s="32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L17" s="16"/>
       <c r="M17" s="17"/>
       <c r="N17" s="18"/>
       <c r="O17" s="13"/>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A18" s="43"/>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="31"/>
       <c r="B18" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="46"/>
-      <c r="D18" s="46">
-        <v>1</v>
-      </c>
-      <c r="E18" s="46"/>
-      <c r="F18" s="46"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="46"/>
-      <c r="I18" s="46"/>
-      <c r="J18" s="46"/>
-      <c r="K18" s="47">
-        <v>1</v>
+      <c r="C18" s="36">
+        <v>1</v>
+      </c>
+      <c r="D18" s="36">
+        <v>2</v>
+      </c>
+      <c r="E18" s="36">
+        <v>1</v>
+      </c>
+      <c r="F18" s="36">
+        <v>1</v>
+      </c>
+      <c r="G18" s="36">
+        <v>1</v>
+      </c>
+      <c r="H18" s="36">
+        <v>1</v>
+      </c>
+      <c r="I18" s="36">
+        <v>1</v>
+      </c>
+      <c r="J18" s="36">
+        <v>1</v>
+      </c>
+      <c r="K18" s="37">
+        <v>2</v>
       </c>
       <c r="L18" s="16">
         <f>SUM(C18:K18)</f>
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="M18" s="17"/>
       <c r="N18" s="18"/>
       <c r="O18" s="13"/>
     </row>
-    <row r="19" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="44"/>
+    <row r="19" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="27"/>
       <c r="B19" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="48">
+      <c r="C19" s="38">
         <f>C17-C18</f>
-        <v>4</v>
-      </c>
-      <c r="D19" s="48">
+        <v>5</v>
+      </c>
+      <c r="D19" s="38">
         <f t="shared" ref="D19:K19" si="4">D17-D18</f>
-        <v>4</v>
-      </c>
-      <c r="E19" s="48">
+        <v>6</v>
+      </c>
+      <c r="E19" s="38">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F19" s="34">
         <f t="shared" si="4"/>
         <v>2</v>
       </c>
-      <c r="G19" s="48">
+      <c r="G19" s="38">
         <f t="shared" si="4"/>
-        <v>5</v>
-      </c>
-      <c r="H19" s="34">
+        <v>7</v>
+      </c>
+      <c r="H19" s="38">
         <f t="shared" si="4"/>
-        <v>3</v>
-      </c>
-      <c r="I19" s="48">
+        <v>5</v>
+      </c>
+      <c r="I19" s="38">
         <f t="shared" si="4"/>
-        <v>3</v>
-      </c>
-      <c r="J19" s="48">
+        <v>5</v>
+      </c>
+      <c r="J19" s="33">
         <f t="shared" si="4"/>
-        <v>5</v>
-      </c>
-      <c r="K19" s="48">
+        <v>3</v>
+      </c>
+      <c r="K19" s="38">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
@@ -1818,15 +1767,15 @@
       <c r="N19" s="18"/>
       <c r="O19" s="21"/>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A20" s="42" t="s">
-        <v>17</v>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="35" t="s">
+        <v>16</v>
       </c>
       <c r="B20" s="28" t="s">
         <v>8</v>
       </c>
       <c r="C20" s="32">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D20" s="32">
         <v>6</v>
@@ -1835,142 +1784,144 @@
         <v>4</v>
       </c>
       <c r="F20" s="32">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G20" s="32">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H20" s="32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I20" s="32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J20" s="32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K20" s="32">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L20" s="16"/>
       <c r="M20" s="17"/>
       <c r="N20" s="18"/>
       <c r="O20" s="13"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A21" s="43"/>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="31"/>
       <c r="B21" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="46">
-        <v>1</v>
-      </c>
-      <c r="D21" s="46">
-        <v>1</v>
-      </c>
-      <c r="E21" s="46">
-        <v>1</v>
-      </c>
-      <c r="F21" s="46"/>
-      <c r="G21" s="46">
-        <v>1</v>
-      </c>
-      <c r="H21" s="46">
-        <v>1</v>
-      </c>
-      <c r="I21" s="46">
-        <v>1</v>
-      </c>
-      <c r="J21" s="46">
-        <v>1</v>
-      </c>
-      <c r="K21" s="47">
-        <v>1</v>
+      <c r="C21" s="36">
+        <v>2</v>
+      </c>
+      <c r="D21" s="36">
+        <v>2</v>
+      </c>
+      <c r="E21" s="36">
+        <v>2</v>
+      </c>
+      <c r="F21" s="36">
+        <v>1</v>
+      </c>
+      <c r="G21" s="36">
+        <v>2</v>
+      </c>
+      <c r="H21" s="36">
+        <v>1</v>
+      </c>
+      <c r="I21" s="36">
+        <v>1</v>
+      </c>
+      <c r="J21" s="36">
+        <v>1</v>
+      </c>
+      <c r="K21" s="37">
+        <v>2</v>
       </c>
       <c r="L21" s="16">
         <f>SUM(C21:K21)</f>
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="M21" s="17"/>
       <c r="N21" s="18"/>
       <c r="O21" s="13"/>
     </row>
-    <row r="22" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="44"/>
+    <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="27"/>
       <c r="B22" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="48">
+      <c r="C22" s="34">
         <f>C20-C21</f>
-        <v>5</v>
-      </c>
-      <c r="D22" s="48">
+        <v>3</v>
+      </c>
+      <c r="D22" s="38">
         <f t="shared" ref="D22:K22" si="5">D20-D21</f>
-        <v>5</v>
-      </c>
-      <c r="E22" s="48">
+        <v>4</v>
+      </c>
+      <c r="E22" s="33">
         <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="F22" s="34">
+        <v>2</v>
+      </c>
+      <c r="F22" s="38">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G22" s="34">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
-      <c r="H22" s="48">
+      <c r="H22" s="38">
         <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="I22" s="48">
+        <v>5</v>
+      </c>
+      <c r="I22" s="38">
         <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-      <c r="J22" s="48">
+        <v>3</v>
+      </c>
+      <c r="J22" s="38">
         <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="K22" s="48">
+        <v>5</v>
+      </c>
+      <c r="K22" s="38">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L22" s="19"/>
       <c r="M22" s="20"/>
       <c r="N22" s="18"/>
       <c r="O22" s="21"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A23" s="42" t="s">
-        <v>18</v>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="35" t="s">
+        <v>17</v>
       </c>
       <c r="B23" s="28" t="s">
         <v>8</v>
       </c>
       <c r="C23" s="32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D23" s="32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E23" s="32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F23" s="32">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G23" s="32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H23" s="32">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I23" s="32">
         <v>4</v>
       </c>
       <c r="J23" s="32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K23" s="32">
         <v>6</v>
@@ -1980,122 +1931,122 @@
       <c r="N23" s="18"/>
       <c r="O23" s="13"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A24" s="43"/>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="31"/>
       <c r="B24" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C24" s="46">
-        <v>1</v>
-      </c>
-      <c r="D24" s="46">
-        <v>2</v>
-      </c>
-      <c r="E24" s="46">
-        <v>1</v>
-      </c>
-      <c r="F24" s="46">
-        <v>1</v>
-      </c>
-      <c r="G24" s="46">
-        <v>1</v>
-      </c>
-      <c r="H24" s="46">
-        <v>1</v>
-      </c>
-      <c r="I24" s="46">
-        <v>1</v>
-      </c>
-      <c r="J24" s="46">
-        <v>1</v>
-      </c>
-      <c r="K24" s="47">
-        <v>1</v>
+      <c r="C24" s="36">
+        <v>2</v>
+      </c>
+      <c r="D24" s="36">
+        <v>2</v>
+      </c>
+      <c r="E24" s="36">
+        <v>2</v>
+      </c>
+      <c r="F24" s="36">
+        <v>1</v>
+      </c>
+      <c r="G24" s="36">
+        <v>2</v>
+      </c>
+      <c r="H24" s="36">
+        <v>1</v>
+      </c>
+      <c r="I24" s="36">
+        <v>1</v>
+      </c>
+      <c r="J24" s="36">
+        <v>1</v>
+      </c>
+      <c r="K24" s="37">
+        <v>2</v>
       </c>
       <c r="L24" s="16">
         <f>SUM(C24:K24)</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="M24" s="17"/>
       <c r="N24" s="18"/>
       <c r="O24" s="13"/>
     </row>
-    <row r="25" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="44"/>
+    <row r="25" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="27"/>
       <c r="B25" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="48">
+      <c r="C25" s="38">
         <f>C23-C24</f>
         <v>4</v>
       </c>
-      <c r="D25" s="48">
+      <c r="D25" s="33">
         <f t="shared" ref="D25:K25" si="6">D23-D24</f>
-        <v>4</v>
-      </c>
-      <c r="E25" s="48">
+        <v>2</v>
+      </c>
+      <c r="E25" s="38">
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="F25" s="48">
+      <c r="F25" s="38">
         <f t="shared" si="6"/>
-        <v>3</v>
-      </c>
-      <c r="G25" s="48">
+        <v>5</v>
+      </c>
+      <c r="G25" s="38">
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="H25" s="34">
+      <c r="H25" s="38">
         <f t="shared" si="6"/>
-        <v>3</v>
-      </c>
-      <c r="I25" s="48">
+        <v>4</v>
+      </c>
+      <c r="I25" s="38">
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
-      <c r="J25" s="48">
+      <c r="J25" s="38">
         <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
-      <c r="K25" s="48">
+        <v>5</v>
+      </c>
+      <c r="K25" s="38">
         <f t="shared" si="6"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L25" s="19"/>
       <c r="M25" s="20"/>
       <c r="N25" s="18"/>
       <c r="O25" s="21"/>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A26" s="42" t="s">
-        <v>19</v>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" s="35" t="s">
+        <v>6</v>
       </c>
       <c r="B26" s="28" t="s">
         <v>8</v>
       </c>
       <c r="C26" s="32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D26" s="32">
         <v>6</v>
       </c>
       <c r="E26" s="32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F26" s="32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G26" s="32">
         <v>4</v>
       </c>
       <c r="H26" s="32">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I26" s="32">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J26" s="32">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K26" s="32">
         <v>6</v>
@@ -2105,64 +2056,62 @@
       <c r="N26" s="18"/>
       <c r="O26" s="13"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="31"/>
       <c r="B27" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C27" s="46">
-        <v>1</v>
-      </c>
-      <c r="D27" s="46">
-        <v>2</v>
-      </c>
-      <c r="E27" s="46">
-        <v>2</v>
-      </c>
-      <c r="F27" s="46">
-        <v>1</v>
-      </c>
-      <c r="G27" s="46">
-        <v>1</v>
-      </c>
-      <c r="H27" s="46">
-        <v>1</v>
-      </c>
-      <c r="I27" s="46">
-        <v>1</v>
-      </c>
-      <c r="J27" s="46">
-        <v>1</v>
-      </c>
-      <c r="K27" s="47">
-        <v>2</v>
+      <c r="C27" s="36">
+        <v>1</v>
+      </c>
+      <c r="D27" s="36">
+        <v>1</v>
+      </c>
+      <c r="E27" s="36">
+        <v>1</v>
+      </c>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36">
+        <v>1</v>
+      </c>
+      <c r="H27" s="36">
+        <v>1</v>
+      </c>
+      <c r="I27" s="36">
+        <v>1</v>
+      </c>
+      <c r="J27" s="36">
+        <v>1</v>
+      </c>
+      <c r="K27" s="37">
+        <v>1</v>
       </c>
       <c r="L27" s="16">
         <f>SUM(C27:K27)</f>
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="M27" s="17"/>
       <c r="N27" s="18"/>
       <c r="O27" s="13"/>
     </row>
-    <row r="28" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="27"/>
       <c r="B28" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C28" s="48">
+      <c r="C28" s="38">
         <f>C26-C27</f>
-        <v>4</v>
-      </c>
-      <c r="D28" s="48">
+        <v>5</v>
+      </c>
+      <c r="D28" s="38">
         <f t="shared" ref="D28:K28" si="7">D26-D27</f>
-        <v>4</v>
-      </c>
-      <c r="E28" s="48">
+        <v>5</v>
+      </c>
+      <c r="E28" s="38">
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
-      <c r="F28" s="48">
+      <c r="F28" s="38">
         <f t="shared" si="7"/>
         <v>4</v>
       </c>
@@ -2170,30 +2119,30 @@
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
-      <c r="H28" s="48">
+      <c r="H28" s="38">
         <f t="shared" si="7"/>
-        <v>4</v>
-      </c>
-      <c r="I28" s="48">
+        <v>7</v>
+      </c>
+      <c r="I28" s="33">
         <f t="shared" si="7"/>
-        <v>2</v>
-      </c>
-      <c r="J28" s="48">
+        <v>1</v>
+      </c>
+      <c r="J28" s="38">
         <f t="shared" si="7"/>
-        <v>4</v>
-      </c>
-      <c r="K28" s="48">
+        <v>7</v>
+      </c>
+      <c r="K28" s="38">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L28" s="19"/>
       <c r="M28" s="20"/>
       <c r="N28" s="18"/>
       <c r="O28" s="21"/>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A29" s="42" t="s">
-        <v>5</v>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" s="35" t="s">
+        <v>18</v>
       </c>
       <c r="B29" s="28" t="s">
         <v>8</v>
@@ -2202,668 +2151,119 @@
         <v>6</v>
       </c>
       <c r="D29" s="32">
+        <v>10</v>
+      </c>
+      <c r="E29" s="32">
         <v>8</v>
       </c>
-      <c r="E29" s="32">
-        <v>6</v>
-      </c>
       <c r="F29" s="32">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G29" s="32">
         <v>8</v>
       </c>
       <c r="H29" s="32">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I29" s="32">
         <v>6</v>
       </c>
       <c r="J29" s="32">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K29" s="32">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L29" s="16"/>
       <c r="M29" s="17"/>
       <c r="N29" s="18"/>
       <c r="O29" s="13"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="31"/>
       <c r="B30" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="46">
-        <v>1</v>
-      </c>
-      <c r="D30" s="46">
-        <v>2</v>
-      </c>
-      <c r="E30" s="46">
-        <v>1</v>
-      </c>
-      <c r="F30" s="46">
-        <v>1</v>
-      </c>
-      <c r="G30" s="46">
-        <v>1</v>
-      </c>
-      <c r="H30" s="46">
-        <v>1</v>
-      </c>
-      <c r="I30" s="46">
-        <v>1</v>
-      </c>
-      <c r="J30" s="46">
-        <v>1</v>
-      </c>
-      <c r="K30" s="47">
-        <v>2</v>
+      <c r="C30" s="36">
+        <v>3</v>
+      </c>
+      <c r="D30" s="36">
+        <v>3</v>
+      </c>
+      <c r="E30" s="36">
+        <v>3</v>
+      </c>
+      <c r="F30" s="36">
+        <v>2</v>
+      </c>
+      <c r="G30" s="36">
+        <v>2</v>
+      </c>
+      <c r="H30" s="36">
+        <v>2</v>
+      </c>
+      <c r="I30" s="36">
+        <v>2</v>
+      </c>
+      <c r="J30" s="36">
+        <v>2</v>
+      </c>
+      <c r="K30" s="37">
+        <v>3</v>
       </c>
       <c r="L30" s="16">
         <f>SUM(C30:K30)</f>
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="M30" s="17"/>
       <c r="N30" s="18"/>
       <c r="O30" s="13"/>
     </row>
-    <row r="31" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="27"/>
       <c r="B31" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="48">
+      <c r="C31" s="38">
         <f>C29-C30</f>
-        <v>5</v>
-      </c>
-      <c r="D31" s="48">
+        <v>3</v>
+      </c>
+      <c r="D31" s="38">
         <f t="shared" ref="D31:K31" si="8">D29-D30</f>
-        <v>6</v>
-      </c>
-      <c r="E31" s="48">
+        <v>7</v>
+      </c>
+      <c r="E31" s="38">
         <f t="shared" si="8"/>
         <v>5</v>
       </c>
-      <c r="F31" s="34">
+      <c r="F31" s="38">
         <f t="shared" si="8"/>
-        <v>2</v>
-      </c>
-      <c r="G31" s="48">
+        <v>4</v>
+      </c>
+      <c r="G31" s="34">
+        <f t="shared" si="8"/>
+        <v>6</v>
+      </c>
+      <c r="H31" s="38">
+        <f t="shared" si="8"/>
+        <v>6</v>
+      </c>
+      <c r="I31" s="33">
+        <f t="shared" si="8"/>
+        <v>4</v>
+      </c>
+      <c r="J31" s="38">
+        <f t="shared" si="8"/>
+        <v>6</v>
+      </c>
+      <c r="K31" s="38">
         <f t="shared" si="8"/>
         <v>7</v>
-      </c>
-      <c r="H31" s="48">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="I31" s="48">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="J31" s="33">
-        <f t="shared" si="8"/>
-        <v>3</v>
-      </c>
-      <c r="K31" s="48">
-        <f t="shared" si="8"/>
-        <v>4</v>
       </c>
       <c r="L31" s="19"/>
       <c r="M31" s="20"/>
       <c r="N31" s="18"/>
       <c r="O31" s="21"/>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A32" s="42" t="s">
-        <v>20</v>
-      </c>
-      <c r="B32" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C32" s="32">
-        <v>5</v>
-      </c>
-      <c r="D32" s="32">
-        <v>6</v>
-      </c>
-      <c r="E32" s="32">
-        <v>4</v>
-      </c>
-      <c r="F32" s="32">
-        <v>5</v>
-      </c>
-      <c r="G32" s="32">
-        <v>5</v>
-      </c>
-      <c r="H32" s="32">
-        <v>6</v>
-      </c>
-      <c r="I32" s="32">
-        <v>4</v>
-      </c>
-      <c r="J32" s="32">
-        <v>6</v>
-      </c>
-      <c r="K32" s="32">
-        <v>7</v>
-      </c>
-      <c r="L32" s="16"/>
-      <c r="M32" s="17"/>
-      <c r="N32" s="18"/>
-      <c r="O32" s="13"/>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A33" s="31"/>
-      <c r="B33" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" s="46">
-        <v>2</v>
-      </c>
-      <c r="D33" s="46">
-        <v>2</v>
-      </c>
-      <c r="E33" s="46">
-        <v>2</v>
-      </c>
-      <c r="F33" s="46">
-        <v>1</v>
-      </c>
-      <c r="G33" s="46">
-        <v>2</v>
-      </c>
-      <c r="H33" s="46">
-        <v>1</v>
-      </c>
-      <c r="I33" s="46">
-        <v>1</v>
-      </c>
-      <c r="J33" s="46">
-        <v>1</v>
-      </c>
-      <c r="K33" s="47">
-        <v>2</v>
-      </c>
-      <c r="L33" s="16">
-        <f>SUM(C33:K33)</f>
-        <v>14</v>
-      </c>
-      <c r="M33" s="17"/>
-      <c r="N33" s="18"/>
-      <c r="O33" s="13"/>
-    </row>
-    <row r="34" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="27"/>
-      <c r="B34" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C34" s="34">
-        <f>C32-C33</f>
-        <v>3</v>
-      </c>
-      <c r="D34" s="48">
-        <f t="shared" ref="D34:K34" si="9">D32-D33</f>
-        <v>4</v>
-      </c>
-      <c r="E34" s="33">
-        <f t="shared" si="9"/>
-        <v>2</v>
-      </c>
-      <c r="F34" s="48">
-        <f t="shared" si="9"/>
-        <v>4</v>
-      </c>
-      <c r="G34" s="34">
-        <f t="shared" si="9"/>
-        <v>3</v>
-      </c>
-      <c r="H34" s="48">
-        <f t="shared" si="9"/>
-        <v>5</v>
-      </c>
-      <c r="I34" s="48">
-        <f t="shared" si="9"/>
-        <v>3</v>
-      </c>
-      <c r="J34" s="48">
-        <f t="shared" si="9"/>
-        <v>5</v>
-      </c>
-      <c r="K34" s="48">
-        <f t="shared" si="9"/>
-        <v>5</v>
-      </c>
-      <c r="L34" s="19"/>
-      <c r="M34" s="20"/>
-      <c r="N34" s="18"/>
-      <c r="O34" s="21"/>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A35" s="42" t="s">
-        <v>21</v>
-      </c>
-      <c r="B35" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C35" s="32">
-        <v>4</v>
-      </c>
-      <c r="D35" s="32">
-        <v>6</v>
-      </c>
-      <c r="E35" s="32">
-        <v>5</v>
-      </c>
-      <c r="F35" s="32">
-        <v>4</v>
-      </c>
-      <c r="G35" s="32">
-        <v>5</v>
-      </c>
-      <c r="H35" s="32">
-        <v>7</v>
-      </c>
-      <c r="I35" s="32">
-        <v>4</v>
-      </c>
-      <c r="J35" s="32">
-        <v>6</v>
-      </c>
-      <c r="K35" s="32">
-        <v>7</v>
-      </c>
-      <c r="L35" s="16"/>
-      <c r="M35" s="17"/>
-      <c r="N35" s="18"/>
-      <c r="O35" s="13"/>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A36" s="31"/>
-      <c r="B36" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C36" s="46">
-        <v>2</v>
-      </c>
-      <c r="D36" s="46">
-        <v>2</v>
-      </c>
-      <c r="E36" s="46">
-        <v>2</v>
-      </c>
-      <c r="F36" s="46">
-        <v>1</v>
-      </c>
-      <c r="G36" s="46">
-        <v>2</v>
-      </c>
-      <c r="H36" s="46">
-        <v>1</v>
-      </c>
-      <c r="I36" s="46">
-        <v>1</v>
-      </c>
-      <c r="J36" s="46">
-        <v>2</v>
-      </c>
-      <c r="K36" s="47">
-        <v>2</v>
-      </c>
-      <c r="L36" s="16">
-        <f>SUM(C36:K36)</f>
-        <v>15</v>
-      </c>
-      <c r="M36" s="17"/>
-      <c r="N36" s="18"/>
-      <c r="O36" s="13"/>
-    </row>
-    <row r="37" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="27"/>
-      <c r="B37" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C37" s="48">
-        <f>C35-C36</f>
-        <v>2</v>
-      </c>
-      <c r="D37" s="48">
-        <f t="shared" ref="D37:K37" si="10">D35-D36</f>
-        <v>4</v>
-      </c>
-      <c r="E37" s="48">
-        <f t="shared" si="10"/>
-        <v>3</v>
-      </c>
-      <c r="F37" s="48">
-        <f t="shared" si="10"/>
-        <v>3</v>
-      </c>
-      <c r="G37" s="34">
-        <f t="shared" si="10"/>
-        <v>3</v>
-      </c>
-      <c r="H37" s="48">
-        <f t="shared" si="10"/>
-        <v>6</v>
-      </c>
-      <c r="I37" s="48">
-        <f t="shared" si="10"/>
-        <v>3</v>
-      </c>
-      <c r="J37" s="48">
-        <f t="shared" si="10"/>
-        <v>4</v>
-      </c>
-      <c r="K37" s="48">
-        <f t="shared" si="10"/>
-        <v>5</v>
-      </c>
-      <c r="L37" s="19"/>
-      <c r="M37" s="20"/>
-      <c r="N37" s="18"/>
-      <c r="O37" s="21"/>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A38" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="B38" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C38" s="32">
-        <v>6</v>
-      </c>
-      <c r="D38" s="45">
-        <v>4</v>
-      </c>
-      <c r="E38" s="32">
-        <v>6</v>
-      </c>
-      <c r="F38" s="32">
-        <v>6</v>
-      </c>
-      <c r="G38" s="32">
-        <v>6</v>
-      </c>
-      <c r="H38" s="32">
-        <v>5</v>
-      </c>
-      <c r="I38" s="32">
-        <v>4</v>
-      </c>
-      <c r="J38" s="32">
-        <v>6</v>
-      </c>
-      <c r="K38" s="32">
-        <v>6</v>
-      </c>
-      <c r="L38" s="16"/>
-      <c r="M38" s="17"/>
-      <c r="N38" s="18"/>
-      <c r="O38" s="13"/>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A39" s="31"/>
-      <c r="B39" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C39" s="46">
-        <v>2</v>
-      </c>
-      <c r="D39" s="46">
-        <v>2</v>
-      </c>
-      <c r="E39" s="46">
-        <v>2</v>
-      </c>
-      <c r="F39" s="46">
-        <v>1</v>
-      </c>
-      <c r="G39" s="46">
-        <v>2</v>
-      </c>
-      <c r="H39" s="46">
-        <v>1</v>
-      </c>
-      <c r="I39" s="46">
-        <v>1</v>
-      </c>
-      <c r="J39" s="46">
-        <v>1</v>
-      </c>
-      <c r="K39" s="47">
-        <v>2</v>
-      </c>
-      <c r="L39" s="16">
-        <f>SUM(C39:K39)</f>
-        <v>14</v>
-      </c>
-      <c r="M39" s="17"/>
-      <c r="N39" s="18"/>
-      <c r="O39" s="13"/>
-    </row>
-    <row r="40" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="27"/>
-      <c r="B40" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C40" s="48">
-        <f>C38-C39</f>
-        <v>4</v>
-      </c>
-      <c r="D40" s="33">
-        <f t="shared" ref="D40:K40" si="11">D38-D39</f>
-        <v>2</v>
-      </c>
-      <c r="E40" s="48">
-        <f t="shared" si="11"/>
-        <v>4</v>
-      </c>
-      <c r="F40" s="48">
-        <f t="shared" si="11"/>
-        <v>5</v>
-      </c>
-      <c r="G40" s="48">
-        <f t="shared" si="11"/>
-        <v>4</v>
-      </c>
-      <c r="H40" s="48">
-        <f t="shared" si="11"/>
-        <v>4</v>
-      </c>
-      <c r="I40" s="48">
-        <f t="shared" si="11"/>
-        <v>3</v>
-      </c>
-      <c r="J40" s="48">
-        <f t="shared" si="11"/>
-        <v>5</v>
-      </c>
-      <c r="K40" s="48">
-        <f t="shared" si="11"/>
-        <v>4</v>
-      </c>
-      <c r="L40" s="19"/>
-      <c r="M40" s="20"/>
-      <c r="N40" s="18"/>
-      <c r="O40" s="21"/>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A41" s="42" t="s">
-        <v>6</v>
-      </c>
-      <c r="B41" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C41" s="32">
-        <v>6</v>
-      </c>
-      <c r="D41" s="32">
-        <v>6</v>
-      </c>
-      <c r="E41" s="32">
-        <v>4</v>
-      </c>
-      <c r="F41" s="32">
-        <v>4</v>
-      </c>
-      <c r="G41" s="32">
-        <v>4</v>
-      </c>
-      <c r="H41" s="32">
-        <v>8</v>
-      </c>
-      <c r="I41" s="32">
-        <v>2</v>
-      </c>
-      <c r="J41" s="32">
-        <v>8</v>
-      </c>
-      <c r="K41" s="32">
-        <v>6</v>
-      </c>
-      <c r="L41" s="16"/>
-      <c r="M41" s="17"/>
-      <c r="N41" s="18"/>
-      <c r="O41" s="13"/>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A42" s="31"/>
-      <c r="B42" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C42" s="46">
-        <v>1</v>
-      </c>
-      <c r="D42" s="46">
-        <v>1</v>
-      </c>
-      <c r="E42" s="46">
-        <v>1</v>
-      </c>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46">
-        <v>1</v>
-      </c>
-      <c r="H42" s="46">
-        <v>1</v>
-      </c>
-      <c r="I42" s="46">
-        <v>1</v>
-      </c>
-      <c r="J42" s="46">
-        <v>1</v>
-      </c>
-      <c r="K42" s="47">
-        <v>1</v>
-      </c>
-      <c r="L42" s="16">
-        <f>SUM(C42:K42)</f>
-        <v>8</v>
-      </c>
-      <c r="M42" s="17"/>
-      <c r="N42" s="18"/>
-      <c r="O42" s="13"/>
-    </row>
-    <row r="43" spans="1:15" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="27"/>
-      <c r="B43" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C43" s="48">
-        <f>C41-C42</f>
-        <v>5</v>
-      </c>
-      <c r="D43" s="48">
-        <f t="shared" ref="D43:K43" si="12">D41-D42</f>
-        <v>5</v>
-      </c>
-      <c r="E43" s="48">
-        <f t="shared" si="12"/>
-        <v>3</v>
-      </c>
-      <c r="F43" s="48">
-        <f t="shared" si="12"/>
-        <v>4</v>
-      </c>
-      <c r="G43" s="34">
-        <f t="shared" si="12"/>
-        <v>3</v>
-      </c>
-      <c r="H43" s="48">
-        <f t="shared" si="12"/>
-        <v>7</v>
-      </c>
-      <c r="I43" s="33">
-        <f t="shared" si="12"/>
-        <v>1</v>
-      </c>
-      <c r="J43" s="48">
-        <f t="shared" si="12"/>
-        <v>7</v>
-      </c>
-      <c r="K43" s="48">
-        <f t="shared" si="12"/>
-        <v>5</v>
-      </c>
-      <c r="L43" s="19"/>
-      <c r="M43" s="20"/>
-      <c r="N43" s="18"/>
-      <c r="O43" s="21"/>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A44" s="50"/>
-      <c r="B44" s="51"/>
-      <c r="C44" s="52"/>
-      <c r="D44" s="52"/>
-      <c r="E44" s="52"/>
-      <c r="F44" s="52"/>
-      <c r="G44" s="52"/>
-      <c r="H44" s="52"/>
-      <c r="I44" s="52"/>
-      <c r="J44" s="52"/>
-      <c r="K44" s="52"/>
-      <c r="L44" s="53"/>
-      <c r="M44" s="54"/>
-      <c r="N44" s="55"/>
-      <c r="O44" s="56"/>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A45" s="36"/>
-      <c r="B45" s="36"/>
-      <c r="C45" s="36"/>
-      <c r="D45" s="36"/>
-      <c r="E45" s="36"/>
-      <c r="F45" s="36"/>
-      <c r="G45" s="36"/>
-      <c r="H45" s="36"/>
-      <c r="I45" s="36"/>
-      <c r="J45" s="36"/>
-      <c r="K45" s="36"/>
-      <c r="N45" s="35">
-        <f>SUM(N10:N28)</f>
-        <v>0</v>
-      </c>
-      <c r="O45" s="35">
-        <f>SUM(O5:O28)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A46" s="36"/>
-      <c r="B46" s="36"/>
-      <c r="C46" s="36"/>
-      <c r="D46" s="36"/>
-      <c r="E46" s="36"/>
-      <c r="F46" s="36"/>
-      <c r="G46" s="36"/>
-      <c r="H46" s="36"/>
-      <c r="I46" s="36"/>
-      <c r="J46" s="36"/>
-      <c r="K46" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
072525 - decrease width of button div/column in skins.ejs....trying to fit cleanly
</commit_message>
<xml_diff>
--- a/public/results/2025/Week 12 Skins.xlsx
+++ b/public/results/2025/Week 12 Skins.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\CODE\golf-league-site\public\results\2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382C94B9-7C59-4F56-9BDD-49ABD9FF6CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{382C94B9-7C59-4F56-9BDD-49ABD9FF6CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9934F819-4F80-4DF6-83E8-7B7EDF157508}"/>
   <bookViews>
-    <workbookView xWindow="555" yWindow="390" windowWidth="19470" windowHeight="10755" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
+    <workbookView xWindow="4635" yWindow="1290" windowWidth="30765" windowHeight="17115" xr2:uid="{F705A57A-943D-4C93-A0B0-17476496A7BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 12 Skins" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="10">
   <si>
     <t>Skins Won</t>
   </si>
@@ -53,12 +53,6 @@
     <t>PAR</t>
   </si>
   <si>
-    <t>Mark Y</t>
-  </si>
-  <si>
-    <t>Mark H</t>
-  </si>
-  <si>
     <t>HDCP</t>
   </si>
   <si>
@@ -71,28 +65,7 @@
     <t>Net</t>
   </si>
   <si>
-    <t>Skins ($40) $4.44/hole</t>
-  </si>
-  <si>
-    <t>Ryan</t>
-  </si>
-  <si>
-    <t>Aaron</t>
-  </si>
-  <si>
-    <t>Matt</t>
-  </si>
-  <si>
-    <t>Tony</t>
-  </si>
-  <si>
-    <t>Mike W</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Shayne I</t>
+    <t>Skins ($xx) $x.xx/hole</t>
   </si>
 </sst>
 </file>
@@ -154,7 +127,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,18 +152,6 @@
         <bgColor rgb="FFD9E2F3"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="25">
     <border>
@@ -523,7 +484,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -618,31 +579,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -659,6 +599,21 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1009,19 +964,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
+      <c r="A1" s="34" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>0</v>
@@ -1065,8 +1020,8 @@
       <c r="K2" s="6">
         <v>9</v>
       </c>
-      <c r="L2" s="43" t="s">
-        <v>7</v>
+      <c r="L2" s="36" t="s">
+        <v>5</v>
       </c>
       <c r="M2" s="7"/>
       <c r="N2" s="8"/>
@@ -1104,7 +1059,7 @@
       <c r="K3" s="11">
         <v>5</v>
       </c>
-      <c r="L3" s="44"/>
+      <c r="L3" s="37"/>
       <c r="M3" s="12"/>
       <c r="N3" s="13"/>
       <c r="O3" s="13"/>
@@ -1112,7 +1067,7 @@
     <row r="4" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="26"/>
       <c r="B4" s="14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C4" s="14">
         <v>4</v>
@@ -1141,45 +1096,25 @@
       <c r="K4" s="15">
         <v>2</v>
       </c>
-      <c r="L4" s="45"/>
+      <c r="L4" s="38"/>
       <c r="M4" s="12"/>
       <c r="N4" s="13"/>
       <c r="O4" s="13"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="35" t="s">
-        <v>12</v>
-      </c>
+      <c r="A5" s="32"/>
       <c r="B5" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="32">
-        <v>5</v>
-      </c>
-      <c r="D5" s="32">
-        <v>9</v>
-      </c>
-      <c r="E5" s="32">
-        <v>5</v>
-      </c>
-      <c r="F5" s="32">
-        <v>3</v>
-      </c>
-      <c r="G5" s="32">
-        <v>4</v>
-      </c>
-      <c r="H5" s="32">
-        <v>5</v>
-      </c>
-      <c r="I5" s="32">
-        <v>4</v>
-      </c>
-      <c r="J5" s="32">
-        <v>5</v>
-      </c>
-      <c r="K5" s="32">
-        <v>7</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="39"/>
+      <c r="I5" s="39"/>
+      <c r="J5" s="39"/>
+      <c r="K5" s="39"/>
       <c r="L5" s="22"/>
       <c r="M5" s="17"/>
       <c r="N5" s="18"/>
@@ -1188,36 +1123,20 @@
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="31"/>
       <c r="B6" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="36">
-        <v>1</v>
-      </c>
-      <c r="D6" s="36">
-        <v>1</v>
-      </c>
-      <c r="E6" s="36">
-        <v>1</v>
-      </c>
-      <c r="F6" s="36"/>
-      <c r="G6" s="36">
-        <v>1</v>
-      </c>
-      <c r="H6" s="36">
-        <v>1</v>
-      </c>
-      <c r="I6" s="36">
-        <v>1</v>
-      </c>
-      <c r="J6" s="36">
-        <v>1</v>
-      </c>
-      <c r="K6" s="37">
-        <v>1</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="40"/>
+      <c r="J6" s="40"/>
+      <c r="K6" s="41"/>
       <c r="L6" s="16">
         <f>SUM(C6:K6)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M6" s="17"/>
       <c r="N6" s="18"/>
@@ -1226,43 +1145,43 @@
     <row r="7" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="27"/>
       <c r="B7" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="38">
+        <v>8</v>
+      </c>
+      <c r="C7" s="42">
         <f>C5-C6</f>
-        <v>4</v>
-      </c>
-      <c r="D7" s="38">
+        <v>0</v>
+      </c>
+      <c r="D7" s="42">
         <f t="shared" ref="D7:K7" si="0">D5-D6</f>
-        <v>8</v>
-      </c>
-      <c r="E7" s="38">
+        <v>0</v>
+      </c>
+      <c r="E7" s="42">
         <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="F7" s="38">
+        <v>0</v>
+      </c>
+      <c r="F7" s="42">
         <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="G7" s="34">
+        <v>0</v>
+      </c>
+      <c r="G7" s="42">
         <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="H7" s="38">
+        <v>0</v>
+      </c>
+      <c r="H7" s="42">
         <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="I7" s="38">
+        <v>0</v>
+      </c>
+      <c r="I7" s="42">
         <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="J7" s="38">
+        <v>0</v>
+      </c>
+      <c r="J7" s="42">
         <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="K7" s="39">
+        <v>0</v>
+      </c>
+      <c r="K7" s="43">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L7" s="19"/>
       <c r="M7" s="17"/>
@@ -1270,39 +1189,19 @@
       <c r="O7" s="13"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="35" t="s">
-        <v>13</v>
-      </c>
+      <c r="A8" s="32"/>
       <c r="B8" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="32">
-        <v>7</v>
-      </c>
-      <c r="D8" s="32">
         <v>6</v>
       </c>
-      <c r="E8" s="32">
-        <v>5</v>
-      </c>
-      <c r="F8" s="32">
-        <v>4</v>
-      </c>
-      <c r="G8" s="32">
-        <v>7</v>
-      </c>
-      <c r="H8" s="32">
-        <v>6</v>
-      </c>
-      <c r="I8" s="32">
-        <v>3</v>
-      </c>
-      <c r="J8" s="32">
-        <v>6</v>
-      </c>
-      <c r="K8" s="32">
-        <v>4</v>
-      </c>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="39"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="39"/>
       <c r="L8" s="22"/>
       <c r="M8" s="17"/>
       <c r="N8" s="18"/>
@@ -1311,38 +1210,20 @@
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="31"/>
       <c r="B9" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="36">
-        <v>1</v>
-      </c>
-      <c r="D9" s="36">
-        <v>1</v>
-      </c>
-      <c r="E9" s="36">
-        <v>1</v>
-      </c>
-      <c r="F9" s="36">
-        <v>1</v>
-      </c>
-      <c r="G9" s="36">
-        <v>1</v>
-      </c>
-      <c r="H9" s="36">
-        <v>1</v>
-      </c>
-      <c r="I9" s="36">
-        <v>1</v>
-      </c>
-      <c r="J9" s="36">
-        <v>1</v>
-      </c>
-      <c r="K9" s="37">
-        <v>1</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C9" s="40"/>
+      <c r="D9" s="40"/>
+      <c r="E9" s="40"/>
+      <c r="F9" s="40"/>
+      <c r="G9" s="40"/>
+      <c r="H9" s="40"/>
+      <c r="I9" s="40"/>
+      <c r="J9" s="40"/>
+      <c r="K9" s="41"/>
       <c r="L9" s="16">
         <f>SUM(C9:K9)</f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="M9" s="17"/>
       <c r="N9" s="18"/>
@@ -1351,43 +1232,43 @@
     <row r="10" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="27"/>
       <c r="B10" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="38">
+        <v>8</v>
+      </c>
+      <c r="C10" s="42">
         <f>C8-C9</f>
-        <v>6</v>
-      </c>
-      <c r="D10" s="38">
+        <v>0</v>
+      </c>
+      <c r="D10" s="42">
         <f t="shared" ref="D10:K10" si="1">D8-D9</f>
-        <v>5</v>
-      </c>
-      <c r="E10" s="38">
+        <v>0</v>
+      </c>
+      <c r="E10" s="42">
         <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="F10" s="38">
+        <v>0</v>
+      </c>
+      <c r="F10" s="42">
         <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="G10" s="38">
+        <v>0</v>
+      </c>
+      <c r="G10" s="42">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="H10" s="38">
+        <v>0</v>
+      </c>
+      <c r="H10" s="42">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="I10" s="38">
+        <v>0</v>
+      </c>
+      <c r="I10" s="42">
         <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="J10" s="38">
+        <v>0</v>
+      </c>
+      <c r="J10" s="42">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K10" s="40">
+        <v>0</v>
+      </c>
+      <c r="K10" s="43">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L10" s="19"/>
       <c r="M10" s="17"/>
@@ -1395,39 +1276,19 @@
       <c r="O10" s="13"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="35" t="s">
-        <v>14</v>
-      </c>
+      <c r="A11" s="32"/>
       <c r="B11" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="32">
         <v>6</v>
       </c>
-      <c r="D11" s="32">
-        <v>6</v>
-      </c>
-      <c r="E11" s="32">
-        <v>4</v>
-      </c>
-      <c r="F11" s="32">
-        <v>2</v>
-      </c>
-      <c r="G11" s="32">
-        <v>4</v>
-      </c>
-      <c r="H11" s="32">
-        <v>5</v>
-      </c>
-      <c r="I11" s="32">
-        <v>3</v>
-      </c>
-      <c r="J11" s="32">
-        <v>5</v>
-      </c>
-      <c r="K11" s="32">
-        <v>5</v>
-      </c>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="39"/>
+      <c r="I11" s="39"/>
+      <c r="J11" s="39"/>
+      <c r="K11" s="39"/>
       <c r="L11" s="16"/>
       <c r="M11" s="17"/>
       <c r="N11" s="18"/>
@@ -1436,36 +1297,20 @@
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="31"/>
       <c r="B12" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="36">
-        <v>1</v>
-      </c>
-      <c r="D12" s="36">
-        <v>1</v>
-      </c>
-      <c r="E12" s="36">
-        <v>1</v>
-      </c>
-      <c r="F12" s="36"/>
-      <c r="G12" s="36">
-        <v>1</v>
-      </c>
-      <c r="H12" s="36">
-        <v>1</v>
-      </c>
-      <c r="I12" s="36">
-        <v>1</v>
-      </c>
-      <c r="J12" s="36">
-        <v>1</v>
-      </c>
-      <c r="K12" s="37">
-        <v>1</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C12" s="40"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="40"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="40"/>
+      <c r="K12" s="41"/>
       <c r="L12" s="16">
         <f>SUM(C12:K12)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M12" s="17"/>
       <c r="N12" s="18"/>
@@ -1474,43 +1319,43 @@
     <row r="13" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="27"/>
       <c r="B13" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="38">
+        <v>8</v>
+      </c>
+      <c r="C13" s="42">
         <f>C11-C12</f>
-        <v>5</v>
-      </c>
-      <c r="D13" s="38">
+        <v>0</v>
+      </c>
+      <c r="D13" s="42">
         <f t="shared" ref="D13:K13" si="2">D11-D12</f>
-        <v>5</v>
-      </c>
-      <c r="E13" s="38">
+        <v>0</v>
+      </c>
+      <c r="E13" s="42">
         <f t="shared" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="F13" s="34">
+        <v>0</v>
+      </c>
+      <c r="F13" s="42">
         <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="G13" s="34">
+        <v>0</v>
+      </c>
+      <c r="G13" s="42">
         <f t="shared" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="H13" s="38">
+        <v>0</v>
+      </c>
+      <c r="H13" s="42">
         <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="I13" s="38">
+        <v>0</v>
+      </c>
+      <c r="I13" s="42">
         <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="J13" s="38">
+        <v>0</v>
+      </c>
+      <c r="J13" s="42">
         <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="K13" s="38">
+        <v>0</v>
+      </c>
+      <c r="K13" s="42">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L13" s="19"/>
       <c r="M13" s="20"/>
@@ -1518,39 +1363,19 @@
       <c r="O13" s="21"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="35" t="s">
-        <v>15</v>
-      </c>
+      <c r="A14" s="32"/>
       <c r="B14" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14" s="32">
-        <v>5</v>
-      </c>
-      <c r="D14" s="32">
         <v>6</v>
       </c>
-      <c r="E14" s="32">
-        <v>5</v>
-      </c>
-      <c r="F14" s="32">
-        <v>5</v>
-      </c>
-      <c r="G14" s="32">
-        <v>4</v>
-      </c>
-      <c r="H14" s="32">
-        <v>5</v>
-      </c>
-      <c r="I14" s="32">
-        <v>3</v>
-      </c>
-      <c r="J14" s="32">
-        <v>5</v>
-      </c>
-      <c r="K14" s="32">
-        <v>6</v>
-      </c>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="39"/>
+      <c r="H14" s="39"/>
+      <c r="I14" s="39"/>
+      <c r="J14" s="39"/>
+      <c r="K14" s="39"/>
       <c r="L14" s="16"/>
       <c r="M14" s="17"/>
       <c r="N14" s="18"/>
@@ -1559,38 +1384,20 @@
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="31"/>
       <c r="B15" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" s="36">
-        <v>1</v>
-      </c>
-      <c r="D15" s="36">
-        <v>2</v>
-      </c>
-      <c r="E15" s="36">
-        <v>2</v>
-      </c>
-      <c r="F15" s="36">
-        <v>1</v>
-      </c>
-      <c r="G15" s="36">
-        <v>1</v>
-      </c>
-      <c r="H15" s="36">
-        <v>1</v>
-      </c>
-      <c r="I15" s="36">
-        <v>1</v>
-      </c>
-      <c r="J15" s="36">
-        <v>1</v>
-      </c>
-      <c r="K15" s="37">
-        <v>2</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="40"/>
+      <c r="I15" s="40"/>
+      <c r="J15" s="40"/>
+      <c r="K15" s="41"/>
       <c r="L15" s="16">
         <f>SUM(C15:K15)</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M15" s="17"/>
       <c r="N15" s="18"/>
@@ -1599,43 +1406,43 @@
     <row r="16" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="27"/>
       <c r="B16" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" s="38">
+        <v>8</v>
+      </c>
+      <c r="C16" s="42">
         <f>C14-C15</f>
-        <v>4</v>
-      </c>
-      <c r="D16" s="38">
+        <v>0</v>
+      </c>
+      <c r="D16" s="42">
         <f t="shared" ref="D16:K16" si="3">D14-D15</f>
-        <v>4</v>
-      </c>
-      <c r="E16" s="38">
+        <v>0</v>
+      </c>
+      <c r="E16" s="42">
         <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-      <c r="F16" s="38">
+        <v>0</v>
+      </c>
+      <c r="F16" s="42">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="G16" s="34">
+        <v>0</v>
+      </c>
+      <c r="G16" s="42">
         <f t="shared" si="3"/>
-        <v>3</v>
-      </c>
-      <c r="H16" s="38">
+        <v>0</v>
+      </c>
+      <c r="H16" s="42">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="I16" s="38">
+        <v>0</v>
+      </c>
+      <c r="I16" s="42">
         <f t="shared" si="3"/>
-        <v>2</v>
-      </c>
-      <c r="J16" s="38">
+        <v>0</v>
+      </c>
+      <c r="J16" s="42">
         <f t="shared" si="3"/>
-        <v>4</v>
-      </c>
-      <c r="K16" s="38">
+        <v>0</v>
+      </c>
+      <c r="K16" s="42">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L16" s="19"/>
       <c r="M16" s="20"/>
@@ -1643,39 +1450,19 @@
       <c r="O16" s="21"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="35" t="s">
-        <v>5</v>
-      </c>
+      <c r="A17" s="32"/>
       <c r="B17" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" s="32">
         <v>6</v>
       </c>
-      <c r="D17" s="32">
-        <v>8</v>
-      </c>
-      <c r="E17" s="32">
-        <v>6</v>
-      </c>
-      <c r="F17" s="32">
-        <v>3</v>
-      </c>
-      <c r="G17" s="32">
-        <v>8</v>
-      </c>
-      <c r="H17" s="32">
-        <v>6</v>
-      </c>
-      <c r="I17" s="32">
-        <v>6</v>
-      </c>
-      <c r="J17" s="32">
-        <v>4</v>
-      </c>
-      <c r="K17" s="32">
-        <v>6</v>
-      </c>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="39"/>
+      <c r="G17" s="39"/>
+      <c r="H17" s="39"/>
+      <c r="I17" s="39"/>
+      <c r="J17" s="39"/>
+      <c r="K17" s="39"/>
       <c r="L17" s="16"/>
       <c r="M17" s="17"/>
       <c r="N17" s="18"/>
@@ -1684,38 +1471,20 @@
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="31"/>
       <c r="B18" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" s="36">
-        <v>1</v>
-      </c>
-      <c r="D18" s="36">
-        <v>2</v>
-      </c>
-      <c r="E18" s="36">
-        <v>1</v>
-      </c>
-      <c r="F18" s="36">
-        <v>1</v>
-      </c>
-      <c r="G18" s="36">
-        <v>1</v>
-      </c>
-      <c r="H18" s="36">
-        <v>1</v>
-      </c>
-      <c r="I18" s="36">
-        <v>1</v>
-      </c>
-      <c r="J18" s="36">
-        <v>1</v>
-      </c>
-      <c r="K18" s="37">
-        <v>2</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="40"/>
+      <c r="K18" s="41"/>
       <c r="L18" s="16">
         <f>SUM(C18:K18)</f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="M18" s="17"/>
       <c r="N18" s="18"/>
@@ -1724,43 +1493,43 @@
     <row r="19" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="27"/>
       <c r="B19" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" s="38">
+        <v>8</v>
+      </c>
+      <c r="C19" s="42">
         <f>C17-C18</f>
-        <v>5</v>
-      </c>
-      <c r="D19" s="38">
+        <v>0</v>
+      </c>
+      <c r="D19" s="42">
         <f t="shared" ref="D19:K19" si="4">D17-D18</f>
-        <v>6</v>
-      </c>
-      <c r="E19" s="38">
+        <v>0</v>
+      </c>
+      <c r="E19" s="42">
         <f t="shared" si="4"/>
-        <v>5</v>
-      </c>
-      <c r="F19" s="34">
+        <v>0</v>
+      </c>
+      <c r="F19" s="42">
         <f t="shared" si="4"/>
-        <v>2</v>
-      </c>
-      <c r="G19" s="38">
+        <v>0</v>
+      </c>
+      <c r="G19" s="42">
         <f t="shared" si="4"/>
-        <v>7</v>
-      </c>
-      <c r="H19" s="38">
+        <v>0</v>
+      </c>
+      <c r="H19" s="42">
         <f t="shared" si="4"/>
-        <v>5</v>
-      </c>
-      <c r="I19" s="38">
+        <v>0</v>
+      </c>
+      <c r="I19" s="42">
         <f t="shared" si="4"/>
-        <v>5</v>
-      </c>
-      <c r="J19" s="33">
+        <v>0</v>
+      </c>
+      <c r="J19" s="42">
         <f t="shared" si="4"/>
-        <v>3</v>
-      </c>
-      <c r="K19" s="38">
+        <v>0</v>
+      </c>
+      <c r="K19" s="42">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L19" s="19"/>
       <c r="M19" s="20"/>
@@ -1768,39 +1537,19 @@
       <c r="O19" s="21"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="35" t="s">
-        <v>16</v>
-      </c>
+      <c r="A20" s="32"/>
       <c r="B20" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="32">
-        <v>5</v>
-      </c>
-      <c r="D20" s="32">
         <v>6</v>
       </c>
-      <c r="E20" s="32">
-        <v>4</v>
-      </c>
-      <c r="F20" s="32">
-        <v>5</v>
-      </c>
-      <c r="G20" s="32">
-        <v>5</v>
-      </c>
-      <c r="H20" s="32">
-        <v>6</v>
-      </c>
-      <c r="I20" s="32">
-        <v>4</v>
-      </c>
-      <c r="J20" s="32">
-        <v>6</v>
-      </c>
-      <c r="K20" s="32">
-        <v>7</v>
-      </c>
+      <c r="C20" s="39"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="39"/>
+      <c r="I20" s="39"/>
+      <c r="J20" s="39"/>
+      <c r="K20" s="39"/>
       <c r="L20" s="16"/>
       <c r="M20" s="17"/>
       <c r="N20" s="18"/>
@@ -1809,38 +1558,20 @@
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="31"/>
       <c r="B21" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" s="36">
-        <v>2</v>
-      </c>
-      <c r="D21" s="36">
-        <v>2</v>
-      </c>
-      <c r="E21" s="36">
-        <v>2</v>
-      </c>
-      <c r="F21" s="36">
-        <v>1</v>
-      </c>
-      <c r="G21" s="36">
-        <v>2</v>
-      </c>
-      <c r="H21" s="36">
-        <v>1</v>
-      </c>
-      <c r="I21" s="36">
-        <v>1</v>
-      </c>
-      <c r="J21" s="36">
-        <v>1</v>
-      </c>
-      <c r="K21" s="37">
-        <v>2</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C21" s="40"/>
+      <c r="D21" s="40"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="40"/>
+      <c r="J21" s="40"/>
+      <c r="K21" s="41"/>
       <c r="L21" s="16">
         <f>SUM(C21:K21)</f>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="M21" s="17"/>
       <c r="N21" s="18"/>
@@ -1849,43 +1580,43 @@
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="27"/>
       <c r="B22" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C22" s="34">
+        <v>8</v>
+      </c>
+      <c r="C22" s="42">
         <f>C20-C21</f>
-        <v>3</v>
-      </c>
-      <c r="D22" s="38">
+        <v>0</v>
+      </c>
+      <c r="D22" s="42">
         <f t="shared" ref="D22:K22" si="5">D20-D21</f>
-        <v>4</v>
-      </c>
-      <c r="E22" s="33">
+        <v>0</v>
+      </c>
+      <c r="E22" s="42">
         <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-      <c r="F22" s="38">
+        <v>0</v>
+      </c>
+      <c r="F22" s="42">
         <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="G22" s="34">
+        <v>0</v>
+      </c>
+      <c r="G22" s="42">
         <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="H22" s="38">
+        <v>0</v>
+      </c>
+      <c r="H22" s="42">
         <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="I22" s="38">
+        <v>0</v>
+      </c>
+      <c r="I22" s="42">
         <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="J22" s="38">
+        <v>0</v>
+      </c>
+      <c r="J22" s="42">
         <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="K22" s="38">
+        <v>0</v>
+      </c>
+      <c r="K22" s="42">
         <f t="shared" si="5"/>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L22" s="19"/>
       <c r="M22" s="20"/>
@@ -1893,39 +1624,19 @@
       <c r="O22" s="21"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="35" t="s">
-        <v>17</v>
-      </c>
+      <c r="A23" s="32"/>
       <c r="B23" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="32">
         <v>6</v>
       </c>
-      <c r="D23" s="32">
-        <v>4</v>
-      </c>
-      <c r="E23" s="32">
-        <v>6</v>
-      </c>
-      <c r="F23" s="32">
-        <v>6</v>
-      </c>
-      <c r="G23" s="32">
-        <v>6</v>
-      </c>
-      <c r="H23" s="32">
-        <v>5</v>
-      </c>
-      <c r="I23" s="32">
-        <v>4</v>
-      </c>
-      <c r="J23" s="32">
-        <v>6</v>
-      </c>
-      <c r="K23" s="32">
-        <v>6</v>
-      </c>
+      <c r="C23" s="39"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="39"/>
+      <c r="I23" s="39"/>
+      <c r="J23" s="39"/>
+      <c r="K23" s="39"/>
       <c r="L23" s="16"/>
       <c r="M23" s="17"/>
       <c r="N23" s="18"/>
@@ -1934,38 +1645,20 @@
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="31"/>
       <c r="B24" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" s="36">
-        <v>2</v>
-      </c>
-      <c r="D24" s="36">
-        <v>2</v>
-      </c>
-      <c r="E24" s="36">
-        <v>2</v>
-      </c>
-      <c r="F24" s="36">
-        <v>1</v>
-      </c>
-      <c r="G24" s="36">
-        <v>2</v>
-      </c>
-      <c r="H24" s="36">
-        <v>1</v>
-      </c>
-      <c r="I24" s="36">
-        <v>1</v>
-      </c>
-      <c r="J24" s="36">
-        <v>1</v>
-      </c>
-      <c r="K24" s="37">
-        <v>2</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="40"/>
+      <c r="J24" s="40"/>
+      <c r="K24" s="41"/>
       <c r="L24" s="16">
         <f>SUM(C24:K24)</f>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="M24" s="17"/>
       <c r="N24" s="18"/>
@@ -1974,43 +1667,43 @@
     <row r="25" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="27"/>
       <c r="B25" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" s="38">
+        <v>8</v>
+      </c>
+      <c r="C25" s="42">
         <f>C23-C24</f>
-        <v>4</v>
-      </c>
-      <c r="D25" s="33">
+        <v>0</v>
+      </c>
+      <c r="D25" s="42">
         <f t="shared" ref="D25:K25" si="6">D23-D24</f>
-        <v>2</v>
-      </c>
-      <c r="E25" s="38">
+        <v>0</v>
+      </c>
+      <c r="E25" s="42">
         <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
-      <c r="F25" s="38">
+        <v>0</v>
+      </c>
+      <c r="F25" s="42">
         <f t="shared" si="6"/>
-        <v>5</v>
-      </c>
-      <c r="G25" s="38">
+        <v>0</v>
+      </c>
+      <c r="G25" s="42">
         <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
-      <c r="H25" s="38">
+        <v>0</v>
+      </c>
+      <c r="H25" s="42">
         <f t="shared" si="6"/>
-        <v>4</v>
-      </c>
-      <c r="I25" s="38">
+        <v>0</v>
+      </c>
+      <c r="I25" s="42">
         <f t="shared" si="6"/>
-        <v>3</v>
-      </c>
-      <c r="J25" s="38">
+        <v>0</v>
+      </c>
+      <c r="J25" s="42">
         <f t="shared" si="6"/>
-        <v>5</v>
-      </c>
-      <c r="K25" s="38">
+        <v>0</v>
+      </c>
+      <c r="K25" s="42">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L25" s="19"/>
       <c r="M25" s="20"/>
@@ -2018,39 +1711,19 @@
       <c r="O25" s="21"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="35" t="s">
+      <c r="A26" s="32"/>
+      <c r="B26" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="B26" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C26" s="32">
-        <v>6</v>
-      </c>
-      <c r="D26" s="32">
-        <v>6</v>
-      </c>
-      <c r="E26" s="32">
-        <v>4</v>
-      </c>
-      <c r="F26" s="32">
-        <v>4</v>
-      </c>
-      <c r="G26" s="32">
-        <v>4</v>
-      </c>
-      <c r="H26" s="32">
-        <v>8</v>
-      </c>
-      <c r="I26" s="32">
-        <v>2</v>
-      </c>
-      <c r="J26" s="32">
-        <v>8</v>
-      </c>
-      <c r="K26" s="32">
-        <v>6</v>
-      </c>
+      <c r="C26" s="39"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="39"/>
+      <c r="I26" s="39"/>
+      <c r="J26" s="39"/>
+      <c r="K26" s="39"/>
       <c r="L26" s="16"/>
       <c r="M26" s="17"/>
       <c r="N26" s="18"/>
@@ -2059,36 +1732,20 @@
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="31"/>
       <c r="B27" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" s="36">
-        <v>1</v>
-      </c>
-      <c r="D27" s="36">
-        <v>1</v>
-      </c>
-      <c r="E27" s="36">
-        <v>1</v>
-      </c>
-      <c r="F27" s="36"/>
-      <c r="G27" s="36">
-        <v>1</v>
-      </c>
-      <c r="H27" s="36">
-        <v>1</v>
-      </c>
-      <c r="I27" s="36">
-        <v>1</v>
-      </c>
-      <c r="J27" s="36">
-        <v>1</v>
-      </c>
-      <c r="K27" s="37">
-        <v>1</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C27" s="40"/>
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40"/>
+      <c r="H27" s="40"/>
+      <c r="I27" s="40"/>
+      <c r="J27" s="40"/>
+      <c r="K27" s="41"/>
       <c r="L27" s="16">
         <f>SUM(C27:K27)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M27" s="17"/>
       <c r="N27" s="18"/>
@@ -2097,43 +1754,43 @@
     <row r="28" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="27"/>
       <c r="B28" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C28" s="38">
+        <v>8</v>
+      </c>
+      <c r="C28" s="42">
         <f>C26-C27</f>
-        <v>5</v>
-      </c>
-      <c r="D28" s="38">
+        <v>0</v>
+      </c>
+      <c r="D28" s="42">
         <f t="shared" ref="D28:K28" si="7">D26-D27</f>
-        <v>5</v>
-      </c>
-      <c r="E28" s="38">
+        <v>0</v>
+      </c>
+      <c r="E28" s="42">
         <f t="shared" si="7"/>
-        <v>3</v>
-      </c>
-      <c r="F28" s="38">
+        <v>0</v>
+      </c>
+      <c r="F28" s="42">
         <f t="shared" si="7"/>
-        <v>4</v>
-      </c>
-      <c r="G28" s="34">
+        <v>0</v>
+      </c>
+      <c r="G28" s="42">
         <f t="shared" si="7"/>
-        <v>3</v>
-      </c>
-      <c r="H28" s="38">
+        <v>0</v>
+      </c>
+      <c r="H28" s="42">
         <f t="shared" si="7"/>
-        <v>7</v>
-      </c>
-      <c r="I28" s="33">
+        <v>0</v>
+      </c>
+      <c r="I28" s="42">
         <f t="shared" si="7"/>
-        <v>1</v>
-      </c>
-      <c r="J28" s="38">
+        <v>0</v>
+      </c>
+      <c r="J28" s="42">
         <f t="shared" si="7"/>
-        <v>7</v>
-      </c>
-      <c r="K28" s="38">
+        <v>0</v>
+      </c>
+      <c r="K28" s="42">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L28" s="19"/>
       <c r="M28" s="20"/>
@@ -2141,39 +1798,19 @@
       <c r="O28" s="21"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="35" t="s">
-        <v>18</v>
-      </c>
+      <c r="A29" s="32"/>
       <c r="B29" s="28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" s="32">
         <v>6</v>
       </c>
-      <c r="D29" s="32">
-        <v>10</v>
-      </c>
-      <c r="E29" s="32">
-        <v>8</v>
-      </c>
-      <c r="F29" s="32">
-        <v>6</v>
-      </c>
-      <c r="G29" s="32">
-        <v>8</v>
-      </c>
-      <c r="H29" s="32">
-        <v>8</v>
-      </c>
-      <c r="I29" s="32">
-        <v>6</v>
-      </c>
-      <c r="J29" s="32">
-        <v>8</v>
-      </c>
-      <c r="K29" s="32">
-        <v>10</v>
-      </c>
+      <c r="C29" s="39"/>
+      <c r="D29" s="39"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="39"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="39"/>
+      <c r="I29" s="39"/>
+      <c r="J29" s="39"/>
+      <c r="K29" s="39"/>
       <c r="L29" s="16"/>
       <c r="M29" s="17"/>
       <c r="N29" s="18"/>
@@ -2182,39 +1819,18 @@
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="31"/>
       <c r="B30" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="C30" s="36">
-        <v>3</v>
-      </c>
-      <c r="D30" s="36">
-        <v>3</v>
-      </c>
-      <c r="E30" s="36">
-        <v>3</v>
-      </c>
-      <c r="F30" s="36">
-        <v>2</v>
-      </c>
-      <c r="G30" s="36">
-        <v>2</v>
-      </c>
-      <c r="H30" s="36">
-        <v>2</v>
-      </c>
-      <c r="I30" s="36">
-        <v>2</v>
-      </c>
-      <c r="J30" s="36">
-        <v>2</v>
-      </c>
-      <c r="K30" s="37">
-        <v>3</v>
-      </c>
-      <c r="L30" s="16">
-        <f>SUM(C30:K30)</f>
-        <v>22</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C30" s="40"/>
+      <c r="D30" s="40"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="40"/>
+      <c r="H30" s="40"/>
+      <c r="I30" s="40"/>
+      <c r="J30" s="40"/>
+      <c r="K30" s="41"/>
+      <c r="L30" s="16"/>
       <c r="M30" s="17"/>
       <c r="N30" s="18"/>
       <c r="O30" s="13"/>
@@ -2222,43 +1838,43 @@
     <row r="31" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="27"/>
       <c r="B31" s="30" t="s">
-        <v>10</v>
-      </c>
-      <c r="C31" s="38">
+        <v>8</v>
+      </c>
+      <c r="C31" s="33">
         <f>C29-C30</f>
-        <v>3</v>
-      </c>
-      <c r="D31" s="38">
+        <v>0</v>
+      </c>
+      <c r="D31" s="33">
         <f t="shared" ref="D31:K31" si="8">D29-D30</f>
-        <v>7</v>
-      </c>
-      <c r="E31" s="38">
+        <v>0</v>
+      </c>
+      <c r="E31" s="33">
         <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="F31" s="38">
+        <v>0</v>
+      </c>
+      <c r="F31" s="33">
         <f t="shared" si="8"/>
-        <v>4</v>
-      </c>
-      <c r="G31" s="34">
+        <v>0</v>
+      </c>
+      <c r="G31" s="42">
         <f t="shared" si="8"/>
-        <v>6</v>
-      </c>
-      <c r="H31" s="38">
+        <v>0</v>
+      </c>
+      <c r="H31" s="42">
         <f t="shared" si="8"/>
-        <v>6</v>
-      </c>
-      <c r="I31" s="33">
+        <v>0</v>
+      </c>
+      <c r="I31" s="42">
         <f t="shared" si="8"/>
-        <v>4</v>
-      </c>
-      <c r="J31" s="38">
+        <v>0</v>
+      </c>
+      <c r="J31" s="42">
         <f t="shared" si="8"/>
-        <v>6</v>
-      </c>
-      <c r="K31" s="38">
+        <v>0</v>
+      </c>
+      <c r="K31" s="33">
         <f t="shared" si="8"/>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L31" s="19"/>
       <c r="M31" s="20"/>

</xml_diff>